<commit_message>
Add Pivot self-serve analysis
</commit_message>
<xml_diff>
--- a/Dashboard/Amazon_Finance_Dashboard_Nandipha.xlsx
+++ b/Dashboard/Amazon_Finance_Dashboard_Nandipha.xlsx
@@ -5,20 +5,35 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0292d34bed0d210/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f0292d34bed0d210/Documents/GitHub/amazon-finance-variance-analysis/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56222C70-AA06-45E3-9D7D-4346B56F0E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{56222C70-AA06-45E3-9D7D-4346B56F0E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E92B1E56-81A4-4FAE-8681-324492D79DCA}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Budget_vs_Actual" sheetId="1" r:id="rId1"/>
     <sheet name="Monthly_Trend" sheetId="2" r:id="rId2"/>
     <sheet name="Executive_Summary" sheetId="3" r:id="rId3"/>
+    <sheet name="Pivot_Analysis" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="Slicer_Category">#N/A</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="4" r:id="rId5"/>
+  </pivotCaches>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
+      <x14:slicerCaches>
+        <x14:slicerCache r:id="rId6"/>
+      </x14:slicerCaches>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
@@ -38,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="26">
   <si>
     <t>Month</t>
   </si>
@@ -95,6 +110,27 @@
   </si>
   <si>
     <t xml:space="preserve">Key Insight: March peak variance 4,5% over budget  driven by Marketing +12,5% Q1 campaign. Other categories under budget offset it. April shows correction -0,7% due to cost control. </t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Column Labels</t>
+  </si>
+  <si>
+    <t>Sum of Variance</t>
+  </si>
+  <si>
+    <t>Total Sum of Variance</t>
+  </si>
+  <si>
+    <t>Total Sum of Variance_%</t>
+  </si>
+  <si>
+    <t>Sum of Variance_%</t>
   </si>
 </sst>
 </file>
@@ -156,13 +192,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1245,6 +1286,465 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>487680</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>99060</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>135255</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Category">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{20C03031-BAE2-8424-49AB-4DBE85BEEEF4}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Category"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4632960" y="1143000"/>
+              <a:ext cx="1828800" cy="2466975"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-ZA" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Sisa Sulelo" refreshedDate="46267.711868171296" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="24" xr:uid="{D50F16CA-54BD-4CB4-99AA-D08BD2A307B2}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:F25" sheet="Budget_vs_Actual"/>
+  </cacheSource>
+  <cacheFields count="6">
+    <cacheField name="Month" numFmtId="0">
+      <sharedItems count="6">
+        <s v="Jan"/>
+        <s v="Feb"/>
+        <s v="Mar"/>
+        <s v="Apr"/>
+        <s v="May"/>
+        <s v="June"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Category" numFmtId="0">
+      <sharedItems count="4">
+        <s v="Marketing"/>
+        <s v="Opertaions"/>
+        <s v="Shipping"/>
+        <s v="Technology"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Budget" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="25000" maxValue="45000"/>
+    </cacheField>
+    <cacheField name="Actual" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="24000" maxValue="50625"/>
+    </cacheField>
+    <cacheField name="Variance" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="-2500" maxValue="5625"/>
+    </cacheField>
+    <cacheField name="Variance_%" numFmtId="10">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="-8.3000000000000004E-2" maxValue="0.125"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition pivotCacheId="703937987"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="24">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="40000"/>
+    <n v="45000"/>
+    <n v="5000"/>
+    <n v="0.125"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="1"/>
+    <n v="30000"/>
+    <n v="28000"/>
+    <n v="-2000"/>
+    <n v="-6.7000000000000004E-2"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <n v="25000"/>
+    <n v="26500"/>
+    <n v="1500"/>
+    <n v="0.06"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="3"/>
+    <n v="35000"/>
+    <n v="34500"/>
+    <n v="-500"/>
+    <n v="-1.4E-2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="40000"/>
+    <n v="42000"/>
+    <n v="2000"/>
+    <n v="0.05"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="30000"/>
+    <n v="31000"/>
+    <n v="1000"/>
+    <n v="3.3000000000000002E-2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <n v="25000"/>
+    <n v="24000"/>
+    <n v="-1000"/>
+    <n v="-0.04"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="3"/>
+    <n v="35000"/>
+    <n v="38000"/>
+    <n v="3000"/>
+    <n v="8.5999999999999993E-2"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="45000"/>
+    <n v="50625"/>
+    <n v="5625"/>
+    <n v="0.125"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="30000"/>
+    <n v="27500"/>
+    <n v="-2500"/>
+    <n v="-8.3000000000000004E-2"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <n v="27000"/>
+    <n v="29000"/>
+    <n v="2000"/>
+    <n v="7.3999999999999996E-2"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="3"/>
+    <n v="35000"/>
+    <n v="36000"/>
+    <n v="1000"/>
+    <n v="2.9000000000000001E-2"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="40000"/>
+    <n v="39500"/>
+    <n v="-500"/>
+    <n v="-1.2999999999999999E-2"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="1"/>
+    <n v="32000"/>
+    <n v="30000"/>
+    <n v="-2000"/>
+    <n v="-6.3E-2"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="2"/>
+    <n v="25000"/>
+    <n v="25500"/>
+    <n v="500"/>
+    <n v="0.02"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <n v="40000"/>
+    <n v="41000"/>
+    <n v="1000"/>
+    <n v="2.5000000000000001E-2"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="0"/>
+    <n v="42000"/>
+    <n v="46000"/>
+    <n v="4000"/>
+    <n v="9.5000000000000001E-2"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="30000"/>
+    <n v="29500"/>
+    <n v="-500"/>
+    <n v="-1.7000000000000001E-2"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="2"/>
+    <n v="26000"/>
+    <n v="25000"/>
+    <n v="-1000"/>
+    <n v="-3.7999999999999999E-2"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="3"/>
+    <n v="35000"/>
+    <n v="33000"/>
+    <n v="-2000"/>
+    <n v="-5.7000000000000002E-2"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="0"/>
+    <n v="40000"/>
+    <n v="43000"/>
+    <n v="3000"/>
+    <n v="7.4999999999999997E-2"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="1"/>
+    <n v="30000"/>
+    <n v="28500"/>
+    <n v="-1500"/>
+    <n v="-0.05"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="2"/>
+    <n v="25000"/>
+    <n v="27000"/>
+    <n v="2000"/>
+    <n v="0.08"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="3"/>
+    <n v="38000"/>
+    <n v="39500"/>
+    <n v="1500"/>
+    <n v="3.9E-2"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4763E40-60D5-41A7-A8C5-FFC2FCD94547}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:O7" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
+  <pivotFields count="6">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="7">
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" numFmtId="10" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="2">
+    <field x="0"/>
+    <field x="-2"/>
+  </colFields>
+  <colItems count="14">
+    <i>
+      <x/>
+      <x/>
+    </i>
+    <i r="1" i="1">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="1"/>
+      <x/>
+    </i>
+    <i r="1" i="1">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+      <x/>
+    </i>
+    <i r="1" i="1">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="3"/>
+      <x/>
+    </i>
+    <i r="1" i="1">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="4"/>
+      <x/>
+    </i>
+    <i r="1" i="1">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="5"/>
+      <x/>
+    </i>
+    <i r="1" i="1">
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+    <i t="grand" i="1">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Sum of Variance" fld="4" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Variance_%" fld="5" baseField="0" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Category" xr10:uid="{F9077A27-98C9-4577-B601-1B5B1053803F}" sourceName="Category">
+  <pivotTables>
+    <pivotTable tabId="4" name="PivotTable1"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="703937987">
+      <items count="4">
+        <i x="0" s="1"/>
+        <i x="1"/>
+        <i x="2"/>
+        <i x="3"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <slicer name="Category" xr10:uid="{E6D5AFD3-2D39-4176-84D9-E2BA2B4EC868}" cache="Slicer_Category" caption="Category" rowHeight="234950"/>
+</slicers>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2201,4 +2701,205 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{975CA393-60A9-43F3-92C8-062AAB44B846}">
+  <dimension ref="A3:O7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B3" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" t="s">
+        <v>14</v>
+      </c>
+      <c r="N4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="8">
+        <v>3000</v>
+      </c>
+      <c r="C6" s="1">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="D6" s="8">
+        <v>5000</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="F6" s="8">
+        <v>2000</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="H6" s="8">
+        <v>5625</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="J6" s="8">
+        <v>-500</v>
+      </c>
+      <c r="K6" s="1">
+        <v>-1.2999999999999999E-2</v>
+      </c>
+      <c r="L6" s="8">
+        <v>4000</v>
+      </c>
+      <c r="M6" s="1">
+        <v>9.5000000000000001E-2</v>
+      </c>
+      <c r="N6" s="8">
+        <v>19125</v>
+      </c>
+      <c r="O6" s="1">
+        <v>0.45699999999999996</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="8">
+        <v>3000</v>
+      </c>
+      <c r="C7" s="1">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="D7" s="8">
+        <v>5000</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="F7" s="8">
+        <v>2000</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="H7" s="8">
+        <v>5625</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="J7" s="8">
+        <v>-500</v>
+      </c>
+      <c r="K7" s="1">
+        <v>-1.2999999999999999E-2</v>
+      </c>
+      <c r="L7" s="8">
+        <v>4000</v>
+      </c>
+      <c r="M7" s="1">
+        <v>9.5000000000000001E-2</v>
+      </c>
+      <c r="N7" s="8">
+        <v>19125</v>
+      </c>
+      <c r="O7" s="1">
+        <v>0.45699999999999996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
+      <x14:slicerList>
+        <x14:slicer r:id="rId3"/>
+      </x14:slicerList>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>